<commit_message>
Página de apresentação (/apresentacao) e ajustes finais da planilha de times
- /apresentacao: 8 telas na ordem do roteiro (problema, dados, ideia, o que o site entrega, por que confiar, valor e
  viabilidade, equipe). O edital pede o "link da apresentação utilizada pela equipe" além do vídeo; esta página é esse link.
  Setas, espaço e rolagem passam de tela; F põe em tela cheia. Os números vêm dos mesmos dados do site.
- Equipe da tela final em TEAM (lib/site.ts). Link "Apresentação" no menu, abaixo de Metodologia.
- Planilha: Tigre Branco → Faculdade Donaduzzi; FATEC PG → Faculdade de Tecnologia de Praia Grande, sigla "FATEC PG".
</commit_message>
<xml_diff>
--- a/para_equipe/nomes_dos_times.xlsx
+++ b/para_equipe/nomes_dos_times.xlsx
@@ -1895,12 +1895,12 @@
       <c r="C41" s="5" t="n"/>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>FATEC PG</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Faculdade de Tecnologia de São Paulo</t>
+          <t>Faculdade de Tecnologia de Praia Grande</t>
         </is>
       </c>
       <c r="F41" s="6" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Faculdade Donaduzz</t>
+          <t>Faculdade Donaduzzi</t>
         </is>
       </c>
       <c r="F57" s="6" t="n">

</xml_diff>